<commit_message>
Caderno de testes: prioridade e casos novos de login, equipe, seleção e campo
</commit_message>
<xml_diff>
--- a/testes/Casos_de_teste_Mulheres_e_Quintais.xlsx
+++ b/testes/Casos_de_teste_Mulheres_e_Quintais.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Resumo" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Casos de teste'!$A$1:$L$66</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Casos de teste'!$A$1:$M$83</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="458">
   <si>
     <t xml:space="preserve">Casos de teste · Sistema Mulheres &amp; Quintais</t>
   </si>
   <si>
-    <t xml:space="preserve">Versão do sistema testada: mq-v95 (setembro de 2026)</t>
+    <t xml:space="preserve">Versão do sistema testada: mq-v97 (setembro de 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Como usar</t>
@@ -39,7 +39,7 @@
     <t xml:space="preserve">1. Cada linha da aba "Casos de teste" é uma coisa para testar. Faça os passos com o perfil indicado e compare com o "Resultado esperado".</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Preencha só as colunas com fundo amarelo: Celular e navegador, Testado por, Data, Resultado e Observação.</t>
+    <t xml:space="preserve">2. A coluna Prioridade diz o que testar primeiro: Crítica, depois Alta, depois Média. Preencha só as colunas com fundo amarelo: Celular e navegador, Testado por, Data, Resultado e Observação.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Em Resultado, escolha: Passou, Falhou, Bloqueado (não deu para testar, por exemplo por falta de pré-condição) ou Não testado.</t>
@@ -90,6 +90,9 @@
     <t xml:space="preserve">Resultado esperado</t>
   </si>
   <si>
+    <t xml:space="preserve">Prioridade</t>
+  </si>
+  <si>
     <t xml:space="preserve">Celular e navegador</t>
   </si>
   <si>
@@ -126,6 +129,9 @@
     <t xml:space="preserve">Aparece o código (ex.: ABCD-2345, vale 7 dias) e a mensagem pronta com endereço, e-mail e código</t>
   </si>
   <si>
+    <t xml:space="preserve">Crítica</t>
+  </si>
+  <si>
     <t xml:space="preserve">Moto G, Chrome</t>
   </si>
   <si>
@@ -210,6 +216,9 @@
     <t xml:space="preserve">Aparece "Este e-mail já tem senha"</t>
   </si>
   <si>
+    <t xml:space="preserve">Alta</t>
+  </si>
+  <si>
     <t xml:space="preserve">A06</t>
   </si>
   <si>
@@ -276,6 +285,9 @@
     <t xml:space="preserve">Volta na mesma aba e na mesma altura da página</t>
   </si>
   <si>
+    <t xml:space="preserve">Média</t>
+  </si>
+  <si>
     <t xml:space="preserve">A10</t>
   </si>
   <si>
@@ -294,6 +306,51 @@
     <t xml:space="preserve">Pede confirmação ("Sair mesmo?") e avisa que só volta a entrar com internet</t>
   </si>
   <si>
+    <t xml:space="preserve">A11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senha errada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pessoa com senha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Já tenho senha → senha errada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"E-mail ou senha incorretos"; não entra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código vencido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código gerado para uma pessoa sem senha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No SQL Editor: update public.acesso_codigos set expira_em = now() - interval '1 minute'; depois tentar o Primeiro acesso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recusado; um código novo funciona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-mail digitado diferente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código recebido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primeiro acesso com o e-mail em maiúsculas ou com espaço no fim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aceita (o sistema ignora maiúsculas e espaços)</t>
+  </si>
+  <si>
     <t xml:space="preserve">C01</t>
   </si>
   <si>
@@ -498,6 +555,63 @@
     <t xml:space="preserve">Mostra a conta; o Histórico registra a consulta com nome e hora</t>
   </si>
   <si>
+    <t xml:space="preserve">C14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editar cadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pessoa ativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ficha → Editar dados → mudar o celular → salvar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celular muda; o CPF não pode ser editado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cadastrar agente de campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agentes de campo → + Agente em PI → cadastrar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agente aparece no cartão do PI, sem limite de vagas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link vencido ou já usado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link já enviado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrir o mesmo link de novo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Link sem validade", com orientação para pedir outro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cadastro fora da sua alçada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Procurar cadastrar professor, auxiliar ou coordenação técnica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os botões não aparecem (só a coordenação geral cadastra)</t>
+  </si>
+  <si>
     <t xml:space="preserve">P01</t>
   </si>
   <si>
@@ -696,6 +810,78 @@
     <t xml:space="preserve">Explica como liberar no celular e deixa explicar o motivo no campo "Sem localização?"</t>
   </si>
   <si>
+    <t xml:space="preserve">S08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sem autorização de uso dos dados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marcar "Não autorizo" no uso dos dados → Salvar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não salva: "Sem a autorização de uso dos dados, a ficha não pode ser registrada"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrigir ficha devolvida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ficha devolvida (S05)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para corrigir → abrir → corrigir → Salvar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volta para "Aguardando aprovação"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lista de espera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichas em lista de espera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ver a lista de espera do estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordenadas pela pontuação de prioridade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baixar planilha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichas lançadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seleção → Baixar planilha (CSV) → abrir no Excel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uma linha por ficha, acentos corretos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dados de outro estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bolsista do PI e fichas da BA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Procurar fichas da BA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não aparecem</t>
+  </si>
+  <si>
     <t xml:space="preserve">F01</t>
   </si>
   <si>
@@ -852,6 +1038,72 @@
     <t xml:space="preserve">Visita aparece como "Atrasada", com o botão do que fazer</t>
   </si>
   <si>
+    <t xml:space="preserve">F11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diagnóstico sem as 3 fotos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salvar com só 1 ou 2 fotos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não salva: pede visão geral, água e plantio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quintal sem água na seca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marcar que a água não dura no período seco → Salvar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não pede plano de kit; conta em "Sem água na seca"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPS sem internet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modo avião, ao ar livre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registra (pode demorar até 1 minuto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancelar visita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visita prevista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrir a visita → Cancelar visita → Confirmar cancelamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some do roteiro de quem ia; o dia de campo volta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrigir plano devolvido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plano devolvido (F06)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para fazer agora → abrir o plano devolvido → corrigir → Salvar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volta para a coordenação aprovar</t>
+  </si>
+  <si>
     <t xml:space="preserve">E01</t>
   </si>
   <si>
@@ -894,9 +1146,6 @@
     <t xml:space="preserve">Não marca mês futuro</t>
   </si>
   <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
     <t xml:space="preserve">No AVA, tentar avançar para o mês seguinte</t>
   </si>
   <si>
@@ -1063,12 +1312,6 @@
   </si>
   <si>
     <t xml:space="preserve">V04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dados de outro estado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bolsista do PI e fichas da BA</t>
   </si>
   <si>
     <t xml:space="preserve">Procurar fichas e pessoas da BA</t>
@@ -1227,16 +1470,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="9"/>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFB23A2E"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFB23A2E"/>
+      <i val="true"/>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1311,7 +1554,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1340,6 +1583,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1364,7 +1611,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1372,7 +1619,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1385,7 +1632,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1405,6 +1652,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB23A2E"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1723,7 +1978,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -1792,7 +2047,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -1801,11 +2056,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1845,1320 +2101,1452 @@
       <c r="L1" s="4" t="s">
         <v>25</v>
       </c>
+      <c r="M1" s="4" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="J2" s="8" t="n">
+      <c r="I2" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="9" t="n">
         <v>46294</v>
       </c>
-      <c r="K2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>36</v>
+      <c r="L2" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
+        <v>44</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="8"/>
       <c r="J3" s="8"/>
-      <c r="K3" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L3" s="7"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
+        <v>50</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="8"/>
       <c r="J4" s="8"/>
-      <c r="K4" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L4" s="7"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M4" s="8"/>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+        <v>56</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="8"/>
       <c r="J5" s="8"/>
-      <c r="K5" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L5" s="7"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
+        <v>62</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6" s="8"/>
       <c r="J6" s="8"/>
-      <c r="K6" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L6" s="7"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
+        <v>68</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L7" s="7"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M7" s="8"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+        <v>74</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" s="8"/>
       <c r="J8" s="8"/>
-      <c r="K8" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L8" s="7"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+        <v>80</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" s="8"/>
       <c r="J9" s="8"/>
-      <c r="K9" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L9" s="7"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M9" s="8"/>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
+        <v>85</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" s="8"/>
       <c r="J10" s="8"/>
-      <c r="K10" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L10" s="7"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M10" s="8"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M11" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M12" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L11" s="7"/>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L12" s="7"/>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>67</v>
-      </c>
       <c r="C13" s="6" t="s">
-        <v>90</v>
+        <v>29</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
+        <v>102</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" s="8"/>
       <c r="J13" s="8"/>
-      <c r="K13" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L13" s="7"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>101</v>
+        <v>40</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>90</v>
+        <v>29</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
+        <v>107</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" s="8"/>
       <c r="J14" s="8"/>
-      <c r="K14" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L14" s="7"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
+        <v>113</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" s="8"/>
       <c r="J15" s="8"/>
-      <c r="K15" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L15" s="7"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
+        <v>118</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I16" s="8"/>
       <c r="J16" s="8"/>
-      <c r="K16" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L16" s="7"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
+        <v>124</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I17" s="8"/>
       <c r="J17" s="8"/>
-      <c r="K17" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L17" s="7"/>
-    </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K17" s="9"/>
+      <c r="L17" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M17" s="8"/>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
+        <v>129</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" s="8"/>
       <c r="J18" s="8"/>
-      <c r="K18" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L18" s="7"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
+        <v>134</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I19" s="8"/>
       <c r="J19" s="8"/>
-      <c r="K19" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L19" s="7"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>101</v>
+        <v>70</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
+        <v>139</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I20" s="8"/>
       <c r="J20" s="8"/>
-      <c r="K20" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L20" s="7"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K20" s="9"/>
+      <c r="L20" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M20" s="8"/>
+    </row>
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
+        <v>144</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I21" s="8"/>
       <c r="J21" s="8"/>
-      <c r="K21" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L21" s="7"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M21" s="8"/>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
+        <v>149</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I22" s="8"/>
       <c r="J22" s="8"/>
-      <c r="K22" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L22" s="7"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
+        <v>154</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I23" s="8"/>
       <c r="J23" s="8"/>
-      <c r="K23" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L23" s="7"/>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K23" s="9"/>
+      <c r="L23" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M23" s="8"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>147</v>
+        <v>70</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
+        <v>159</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I24" s="8"/>
       <c r="J24" s="8"/>
-      <c r="K24" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L24" s="7"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M24" s="8"/>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
+        <v>164</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I25" s="8"/>
       <c r="J25" s="8"/>
-      <c r="K25" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L25" s="7"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M25" s="8"/>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>84</v>
+        <v>166</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
+        <v>170</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I26" s="8"/>
       <c r="J26" s="8"/>
-      <c r="K26" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L26" s="7"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M26" s="8"/>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>84</v>
+        <v>166</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
+        <v>175</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I27" s="8"/>
       <c r="J27" s="8"/>
-      <c r="K27" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L27" s="7"/>
-    </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K27" s="9"/>
+      <c r="L27" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M27" s="8"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>173</v>
+        <v>70</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
+        <v>180</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I28" s="8"/>
       <c r="J28" s="8"/>
-      <c r="K28" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L28" s="7"/>
-    </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K28" s="9"/>
+      <c r="L28" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M28" s="8"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>179</v>
+        <v>70</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="H29" s="7"/>
-      <c r="I29" s="7"/>
+        <v>185</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I29" s="8"/>
       <c r="J29" s="8"/>
-      <c r="K29" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L29" s="7"/>
-    </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K29" s="9"/>
+      <c r="L29" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M29" s="8"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>179</v>
+        <v>120</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>56</v>
+        <v>188</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
+        <v>190</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I30" s="8"/>
       <c r="J30" s="8"/>
-      <c r="K30" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L30" s="7"/>
+      <c r="K30" s="9"/>
+      <c r="L30" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M30" s="8"/>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>189</v>
+        <v>109</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
+        <v>194</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I31" s="8"/>
       <c r="J31" s="8"/>
-      <c r="K31" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L31" s="7"/>
-    </row>
-    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K31" s="9"/>
+      <c r="L31" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M31" s="8"/>
+    </row>
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D32" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="9"/>
+      <c r="L32" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M32" s="8"/>
+    </row>
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="E33" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="H32" s="7"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="8"/>
-      <c r="K32" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L32" s="7"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>200</v>
-      </c>
       <c r="F33" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
+        <v>204</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I33" s="8"/>
       <c r="J33" s="8"/>
-      <c r="K33" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L33" s="7"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M33" s="8"/>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
+        <v>209</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I34" s="8"/>
       <c r="J34" s="8"/>
-      <c r="K34" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L34" s="7"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M34" s="8"/>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>67</v>
+        <v>211</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="H35" s="7"/>
-      <c r="I35" s="7"/>
+        <v>215</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I35" s="8"/>
       <c r="J35" s="8"/>
-      <c r="K35" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L35" s="7"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M35" s="8"/>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>67</v>
+        <v>217</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
+        <v>221</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I36" s="8"/>
       <c r="J36" s="8"/>
-      <c r="K36" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L36" s="7"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M36" s="8"/>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>84</v>
+        <v>217</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>220</v>
+        <v>58</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
+        <v>225</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I37" s="8"/>
       <c r="J37" s="8"/>
-      <c r="K37" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L37" s="7"/>
+      <c r="K37" s="9"/>
+      <c r="L37" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M37" s="8"/>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F38" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I38" s="8"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="9"/>
+      <c r="L38" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M38" s="8"/>
+    </row>
+    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="G38" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
-      <c r="J38" s="8"/>
-      <c r="K38" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L38" s="7"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="D39" s="6" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>231</v>
+        <v>90</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="H39" s="7"/>
-      <c r="I39" s="7"/>
+        <v>235</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I39" s="8"/>
       <c r="J39" s="8"/>
-      <c r="K39" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L39" s="7"/>
-    </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K39" s="9"/>
+      <c r="L39" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M39" s="8"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>235</v>
+        <v>88</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="H40" s="7"/>
-      <c r="I40" s="7"/>
+        <v>240</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I40" s="8"/>
       <c r="J40" s="8"/>
-      <c r="K40" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L40" s="7"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K40" s="9"/>
+      <c r="L40" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M40" s="8"/>
+    </row>
+    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>235</v>
+        <v>88</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="H41" s="7"/>
-      <c r="I41" s="7"/>
+        <v>245</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I41" s="8"/>
       <c r="J41" s="8"/>
-      <c r="K41" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L41" s="7"/>
+      <c r="K41" s="9"/>
+      <c r="L41" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M41" s="8"/>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>235</v>
+        <v>70</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="H42" s="7"/>
-      <c r="I42" s="7"/>
+        <v>250</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I42" s="8"/>
       <c r="J42" s="8"/>
-      <c r="K42" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L42" s="7"/>
+      <c r="K42" s="9"/>
+      <c r="L42" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M42" s="8"/>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="H43" s="7"/>
-      <c r="I43" s="7"/>
+        <v>255</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I43" s="8"/>
       <c r="J43" s="8"/>
-      <c r="K43" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L43" s="7"/>
+      <c r="K43" s="9"/>
+      <c r="L43" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M43" s="8"/>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>235</v>
+        <v>88</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="H44" s="7"/>
-      <c r="I44" s="7"/>
+        <v>260</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I44" s="8"/>
       <c r="J44" s="8"/>
-      <c r="K44" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L44" s="7"/>
+      <c r="K44" s="9"/>
+      <c r="L44" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M44" s="8"/>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>235</v>
+        <v>88</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>262</v>
+        <v>238</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>263</v>
@@ -3166,23 +3554,26 @@
       <c r="G45" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="H45" s="7"/>
-      <c r="I45" s="7"/>
+      <c r="H45" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I45" s="8"/>
       <c r="J45" s="8"/>
-      <c r="K45" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L45" s="7"/>
+      <c r="K45" s="9"/>
+      <c r="L45" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M45" s="8"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
         <v>265</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>235</v>
+        <v>88</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>266</v>
@@ -3196,23 +3587,26 @@
       <c r="G46" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="H46" s="7"/>
-      <c r="I46" s="7"/>
+      <c r="H46" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I46" s="8"/>
       <c r="J46" s="8"/>
-      <c r="K46" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L46" s="7"/>
-    </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K46" s="9"/>
+      <c r="L46" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M46" s="8"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
         <v>270</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>271</v>
@@ -3226,389 +3620,428 @@
       <c r="G47" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="H47" s="7"/>
-      <c r="I47" s="7"/>
+      <c r="H47" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I47" s="8"/>
       <c r="J47" s="8"/>
-      <c r="K47" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L47" s="7"/>
-    </row>
-    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K47" s="9"/>
+      <c r="L47" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M47" s="8"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
         <v>275</v>
       </c>
       <c r="B48" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="E48" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="F48" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="E48" s="6" t="s">
+      <c r="G48" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="F48" s="6" t="s">
+      <c r="H48" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I48" s="8"/>
+      <c r="J48" s="8"/>
+      <c r="K48" s="9"/>
+      <c r="L48" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M48" s="8"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="G48" s="6" t="s">
+      <c r="B49" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D49" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="H48" s="7"/>
-      <c r="I48" s="7"/>
-      <c r="J48" s="8"/>
-      <c r="K48" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L48" s="7"/>
-    </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="s">
+      <c r="E49" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="B49" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="D49" s="6" t="s">
+      <c r="F49" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="G49" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="F49" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="G49" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="H49" s="7"/>
-      <c r="I49" s="7"/>
+      <c r="H49" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I49" s="8"/>
       <c r="J49" s="8"/>
-      <c r="K49" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L49" s="7"/>
+      <c r="K49" s="9"/>
+      <c r="L49" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M49" s="8"/>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="B50" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="D50" s="6" t="s">
+      <c r="E50" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="E50" s="6" t="s">
+      <c r="F50" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="F50" s="6" t="s">
+      <c r="G50" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="G50" s="6" t="s">
+      <c r="H50" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I50" s="8"/>
+      <c r="J50" s="8"/>
+      <c r="K50" s="9"/>
+      <c r="L50" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M50" s="8"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="H50" s="7"/>
-      <c r="I50" s="7"/>
-      <c r="J50" s="8"/>
-      <c r="K50" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L50" s="7"/>
-    </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="s">
+      <c r="B51" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D51" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="B51" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="D51" s="6" t="s">
+      <c r="E51" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="F51" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="F51" s="6" t="s">
+      <c r="G51" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="G51" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="H51" s="7"/>
-      <c r="I51" s="7"/>
+      <c r="H51" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I51" s="8"/>
       <c r="J51" s="8"/>
-      <c r="K51" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L51" s="7"/>
+      <c r="K51" s="9"/>
+      <c r="L51" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M51" s="8"/>
     </row>
     <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="B52" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="B52" s="6" t="s">
-        <v>84</v>
-      </c>
       <c r="C52" s="6" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>298</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>289</v>
+        <v>299</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="H52" s="7"/>
-      <c r="I52" s="7"/>
+        <v>301</v>
+      </c>
+      <c r="H52" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I52" s="8"/>
       <c r="J52" s="8"/>
-      <c r="K52" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L52" s="7"/>
-    </row>
-    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K52" s="9"/>
+      <c r="L52" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M52" s="8"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>84</v>
+        <v>297</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>303</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>191</v>
+        <v>304</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="H53" s="7"/>
-      <c r="I53" s="7"/>
+        <v>306</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I53" s="8"/>
       <c r="J53" s="8"/>
-      <c r="K53" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L53" s="7"/>
+      <c r="K53" s="9"/>
+      <c r="L53" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M53" s="8"/>
     </row>
     <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>84</v>
+        <v>297</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>310</v>
-      </c>
-      <c r="H54" s="7"/>
-      <c r="I54" s="7"/>
+        <v>311</v>
+      </c>
+      <c r="H54" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I54" s="8"/>
       <c r="J54" s="8"/>
-      <c r="K54" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L54" s="7"/>
+      <c r="K54" s="9"/>
+      <c r="L54" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M54" s="8"/>
     </row>
     <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>173</v>
+        <v>70</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>294</v>
+        <v>314</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>314</v>
-      </c>
-      <c r="H55" s="7"/>
-      <c r="I55" s="7"/>
+        <v>316</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I55" s="8"/>
       <c r="J55" s="8"/>
-      <c r="K55" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L55" s="7"/>
+      <c r="K55" s="9"/>
+      <c r="L55" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M55" s="8"/>
     </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>67</v>
+        <v>297</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>319</v>
-      </c>
-      <c r="H56" s="7"/>
-      <c r="I56" s="7"/>
+        <v>321</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I56" s="8"/>
       <c r="J56" s="8"/>
-      <c r="K56" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L56" s="7"/>
+      <c r="K56" s="9"/>
+      <c r="L56" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M56" s="8"/>
     </row>
     <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>27</v>
+        <v>297</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="H57" s="7"/>
-      <c r="I57" s="7"/>
+        <v>326</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I57" s="8"/>
       <c r="J57" s="8"/>
-      <c r="K57" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L57" s="7"/>
-    </row>
-    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K57" s="9"/>
+      <c r="L57" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M57" s="8"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>147</v>
+        <v>297</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>329</v>
-      </c>
-      <c r="H58" s="7"/>
-      <c r="I58" s="7"/>
+        <v>331</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I58" s="8"/>
       <c r="J58" s="8"/>
-      <c r="K58" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L58" s="7"/>
+      <c r="K58" s="9"/>
+      <c r="L58" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M58" s="8"/>
     </row>
     <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>331</v>
+        <v>286</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>335</v>
-      </c>
-      <c r="H59" s="7"/>
-      <c r="I59" s="7"/>
+        <v>336</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I59" s="8"/>
       <c r="J59" s="8"/>
-      <c r="K59" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L59" s="7"/>
-    </row>
-    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K59" s="9"/>
+      <c r="L59" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M59" s="8"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>27</v>
+        <v>297</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>331</v>
+        <v>286</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>338</v>
+        <v>304</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>339</v>
@@ -3616,29 +4049,32 @@
       <c r="G60" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="H60" s="7"/>
-      <c r="I60" s="7"/>
+      <c r="H60" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I60" s="8"/>
       <c r="J60" s="8"/>
-      <c r="K60" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L60" s="7"/>
-    </row>
-    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K60" s="9"/>
+      <c r="L60" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M60" s="8"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
         <v>341</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>27</v>
+        <v>297</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>331</v>
+        <v>286</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>342</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>289</v>
+        <v>304</v>
       </c>
       <c r="F61" s="6" t="s">
         <v>343</v>
@@ -3646,23 +4082,26 @@
       <c r="G61" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="H61" s="7"/>
-      <c r="I61" s="7"/>
+      <c r="H61" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I61" s="8"/>
       <c r="J61" s="8"/>
-      <c r="K61" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L61" s="7"/>
-    </row>
-    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K61" s="9"/>
+      <c r="L61" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M61" s="8"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
         <v>345</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>84</v>
+        <v>297</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>331</v>
+        <v>286</v>
       </c>
       <c r="D62" s="6" t="s">
         <v>346</v>
@@ -3671,34 +4110,37 @@
         <v>347</v>
       </c>
       <c r="F62" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="G62" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="G62" s="6" t="s">
-        <v>349</v>
-      </c>
-      <c r="H62" s="7"/>
-      <c r="I62" s="7"/>
+      <c r="H62" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I62" s="8"/>
       <c r="J62" s="8"/>
-      <c r="K62" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L62" s="7"/>
+      <c r="K62" s="9"/>
+      <c r="L62" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M62" s="8"/>
     </row>
     <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D63" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="B63" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>331</v>
-      </c>
-      <c r="D63" s="6" t="s">
+      <c r="E63" s="6" t="s">
         <v>351</v>
-      </c>
-      <c r="E63" s="6" t="s">
-        <v>289</v>
       </c>
       <c r="F63" s="6" t="s">
         <v>352</v>
@@ -3706,23 +4148,26 @@
       <c r="G63" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="H63" s="7"/>
-      <c r="I63" s="7"/>
+      <c r="H63" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I63" s="8"/>
       <c r="J63" s="8"/>
-      <c r="K63" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L63" s="7"/>
+      <c r="K63" s="9"/>
+      <c r="L63" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M63" s="8"/>
     </row>
     <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
         <v>354</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>179</v>
+        <v>297</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>331</v>
+        <v>286</v>
       </c>
       <c r="D64" s="6" t="s">
         <v>355</v>
@@ -3736,89 +4181,659 @@
       <c r="G64" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="H64" s="7"/>
-      <c r="I64" s="7"/>
+      <c r="H64" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I64" s="8"/>
       <c r="J64" s="8"/>
-      <c r="K64" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L64" s="7"/>
+      <c r="K64" s="9"/>
+      <c r="L64" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M64" s="8"/>
     </row>
     <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
         <v>359</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>179</v>
+        <v>360</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>331</v>
+        <v>361</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>363</v>
-      </c>
-      <c r="H65" s="7"/>
-      <c r="I65" s="7"/>
+        <v>365</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I65" s="8"/>
       <c r="J65" s="8"/>
-      <c r="K65" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L65" s="7"/>
+      <c r="K65" s="9"/>
+      <c r="L65" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M65" s="8"/>
     </row>
     <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>179</v>
+        <v>360</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>331</v>
+        <v>361</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="H66" s="7"/>
-      <c r="I66" s="7"/>
+        <v>370</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I66" s="8"/>
       <c r="J66" s="8"/>
-      <c r="K66" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L66" s="7"/>
+      <c r="K66" s="9"/>
+      <c r="L66" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M66" s="8"/>
+    </row>
+    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="H67" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I67" s="8"/>
+      <c r="J67" s="8"/>
+      <c r="K67" s="9"/>
+      <c r="L67" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M67" s="8"/>
+    </row>
+    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="G68" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I68" s="8"/>
+      <c r="J68" s="8"/>
+      <c r="K68" s="9"/>
+      <c r="L68" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M68" s="8"/>
+    </row>
+    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="G69" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I69" s="8"/>
+      <c r="J69" s="8"/>
+      <c r="K69" s="9"/>
+      <c r="L69" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M69" s="8"/>
+    </row>
+    <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I70" s="8"/>
+      <c r="J70" s="8"/>
+      <c r="K70" s="9"/>
+      <c r="L70" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M70" s="8"/>
+    </row>
+    <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="G71" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="H71" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I71" s="8"/>
+      <c r="J71" s="8"/>
+      <c r="K71" s="9"/>
+      <c r="L71" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M71" s="8"/>
+    </row>
+    <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="G72" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I72" s="8"/>
+      <c r="J72" s="8"/>
+      <c r="K72" s="9"/>
+      <c r="L72" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M72" s="8"/>
+    </row>
+    <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="G73" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="H73" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I73" s="8"/>
+      <c r="J73" s="8"/>
+      <c r="K73" s="9"/>
+      <c r="L73" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M73" s="8"/>
+    </row>
+    <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="G74" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I74" s="8"/>
+      <c r="J74" s="8"/>
+      <c r="K74" s="9"/>
+      <c r="L74" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M74" s="8"/>
+    </row>
+    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="G75" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I75" s="8"/>
+      <c r="J75" s="8"/>
+      <c r="K75" s="9"/>
+      <c r="L75" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M75" s="8"/>
+    </row>
+    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="G76" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I76" s="8"/>
+      <c r="J76" s="8"/>
+      <c r="K76" s="9"/>
+      <c r="L76" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M76" s="8"/>
+    </row>
+    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="G77" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="H77" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I77" s="8"/>
+      <c r="J77" s="8"/>
+      <c r="K77" s="9"/>
+      <c r="L77" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M77" s="8"/>
+    </row>
+    <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="G78" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I78" s="8"/>
+      <c r="J78" s="8"/>
+      <c r="K78" s="9"/>
+      <c r="L78" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M78" s="8"/>
+    </row>
+    <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="G79" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="H79" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I79" s="8"/>
+      <c r="J79" s="8"/>
+      <c r="K79" s="9"/>
+      <c r="L79" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M79" s="8"/>
+    </row>
+    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="G80" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I80" s="8"/>
+      <c r="J80" s="8"/>
+      <c r="K80" s="9"/>
+      <c r="L80" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M80" s="8"/>
+    </row>
+    <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="G81" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="H81" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I81" s="8"/>
+      <c r="J81" s="8"/>
+      <c r="K81" s="9"/>
+      <c r="L81" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M81" s="8"/>
+    </row>
+    <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="H82" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I82" s="8"/>
+      <c r="J82" s="8"/>
+      <c r="K82" s="9"/>
+      <c r="L82" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M82" s="8"/>
+    </row>
+    <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="G83" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I83" s="8"/>
+      <c r="J83" s="8"/>
+      <c r="K83" s="9"/>
+      <c r="L83" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M83" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L66"/>
-  <conditionalFormatting sqref="K2:K66">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
-      <formula>$K2="Passou"</formula>
+  <autoFilter ref="A1:M83"/>
+  <conditionalFormatting sqref="L2:L83">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+      <formula>$L2="Passou"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
-      <formula>$K2="Falhou"</formula>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>$L2="Falhou"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
-      <formula>$K2="Bloqueado"</formula>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Escolha Passou, Falhou, Bloqueado ou Não testado." errorStyle="stop" errorTitle="Resultado" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K66" type="list">
+    <dataValidation allowBlank="true" error="Escolha Passou, Falhou, Bloqueado ou Não testado." errorStyle="stop" errorTitle="Resultado" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L83" type="list">
       <formula1>"Passou,Falhou,Bloqueado,Não testado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3855,335 +4870,335 @@
         <v>16</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>369</v>
+        <v>450</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>370</v>
+        <v>451</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>371</v>
+        <v>452</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>372</v>
+        <v>453</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>373</v>
+        <v>454</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="9" t="n">
-        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$66,A2)</f>
-        <v>10</v>
-      </c>
-      <c r="C2" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A2,'Casos de teste'!$K$2:$K$66,"Passou")</f>
+      <c r="A2" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="10" t="n">
+        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$83,A2)</f>
+        <v>13</v>
+      </c>
+      <c r="C2" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A2,'Casos de teste'!$L$2:$L$83,"Passou")</f>
         <v>1</v>
       </c>
-      <c r="D2" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A2,'Casos de teste'!$K$2:$K$66,"Falhou")</f>
+      <c r="D2" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A2,'Casos de teste'!$L$2:$L$83,"Falhou")</f>
         <v>0</v>
       </c>
-      <c r="E2" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A2,'Casos de teste'!$K$2:$K$66,"Bloqueado")</f>
+      <c r="E2" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A2,'Casos de teste'!$L$2:$L$83,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="F2" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A2,'Casos de teste'!$K$2:$K$66,"Não testado")</f>
-        <v>9</v>
-      </c>
-      <c r="G2" s="10" t="n">
+      <c r="F2" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A2,'Casos de teste'!$L$2:$L$83,"Não testado")</f>
+        <v>12</v>
+      </c>
+      <c r="G2" s="11" t="n">
         <f aca="false">IF(B2=0,0,(C2+D2)/B2)</f>
-        <v>0.1</v>
-      </c>
-      <c r="H2" s="10" t="n">
+        <v>0.0769230769230769</v>
+      </c>
+      <c r="H2" s="11" t="n">
         <f aca="false">IF(C2+D2=0,"-",C2/(C2+D2))</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="B3" s="9" t="n">
-        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$66,A3)</f>
-        <v>13</v>
-      </c>
-      <c r="C3" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A3,'Casos de teste'!$K$2:$K$66,"Passou")</f>
+      <c r="A3" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" s="10" t="n">
+        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$83,A3)</f>
+        <v>17</v>
+      </c>
+      <c r="C3" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A3,'Casos de teste'!$L$2:$L$83,"Passou")</f>
         <v>0</v>
       </c>
-      <c r="D3" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A3,'Casos de teste'!$K$2:$K$66,"Falhou")</f>
+      <c r="D3" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A3,'Casos de teste'!$L$2:$L$83,"Falhou")</f>
         <v>0</v>
       </c>
-      <c r="E3" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A3,'Casos de teste'!$K$2:$K$66,"Bloqueado")</f>
+      <c r="E3" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A3,'Casos de teste'!$L$2:$L$83,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A3,'Casos de teste'!$K$2:$K$66,"Não testado")</f>
-        <v>13</v>
-      </c>
-      <c r="G3" s="10" t="n">
+      <c r="F3" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A3,'Casos de teste'!$L$2:$L$83,"Não testado")</f>
+        <v>17</v>
+      </c>
+      <c r="G3" s="11" t="n">
         <f aca="false">IF(B3=0,0,(C3+D3)/B3)</f>
         <v>0</v>
       </c>
-      <c r="H3" s="10" t="str">
+      <c r="H3" s="11" t="str">
         <f aca="false">IF(C3+D3=0,"-",C3/(C3+D3))</f>
         <v>-</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="B4" s="9" t="n">
-        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$66,A4)</f>
+      <c r="A4" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="B4" s="10" t="n">
+        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$83,A4)</f>
         <v>6</v>
       </c>
-      <c r="C4" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A4,'Casos de teste'!$K$2:$K$66,"Passou")</f>
+      <c r="C4" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A4,'Casos de teste'!$L$2:$L$83,"Passou")</f>
         <v>0</v>
       </c>
-      <c r="D4" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A4,'Casos de teste'!$K$2:$K$66,"Falhou")</f>
+      <c r="D4" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A4,'Casos de teste'!$L$2:$L$83,"Falhou")</f>
         <v>0</v>
       </c>
-      <c r="E4" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A4,'Casos de teste'!$K$2:$K$66,"Bloqueado")</f>
+      <c r="E4" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A4,'Casos de teste'!$L$2:$L$83,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A4,'Casos de teste'!$K$2:$K$66,"Não testado")</f>
+      <c r="F4" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A4,'Casos de teste'!$L$2:$L$83,"Não testado")</f>
         <v>6</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="G4" s="11" t="n">
         <f aca="false">IF(B4=0,0,(C4+D4)/B4)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="10" t="str">
+      <c r="H4" s="11" t="str">
         <f aca="false">IF(C4+D4=0,"-",C4/(C4+D4))</f>
         <v>-</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="B5" s="9" t="n">
-        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$66,A5)</f>
-        <v>7</v>
-      </c>
-      <c r="C5" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A5,'Casos de teste'!$K$2:$K$66,"Passou")</f>
+      <c r="A5" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B5" s="10" t="n">
+        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$83,A5)</f>
+        <v>12</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A5,'Casos de teste'!$L$2:$L$83,"Passou")</f>
         <v>0</v>
       </c>
-      <c r="D5" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A5,'Casos de teste'!$K$2:$K$66,"Falhou")</f>
+      <c r="D5" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A5,'Casos de teste'!$L$2:$L$83,"Falhou")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A5,'Casos de teste'!$K$2:$K$66,"Bloqueado")</f>
+      <c r="E5" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A5,'Casos de teste'!$L$2:$L$83,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="F5" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A5,'Casos de teste'!$K$2:$K$66,"Não testado")</f>
-        <v>7</v>
-      </c>
-      <c r="G5" s="10" t="n">
+      <c r="F5" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A5,'Casos de teste'!$L$2:$L$83,"Não testado")</f>
+        <v>12</v>
+      </c>
+      <c r="G5" s="11" t="n">
         <f aca="false">IF(B5=0,0,(C5+D5)/B5)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="10" t="str">
+      <c r="H5" s="11" t="str">
         <f aca="false">IF(C5+D5=0,"-",C5/(C5+D5))</f>
         <v>-</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="B6" s="9" t="n">
-        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$66,A6)</f>
-        <v>10</v>
-      </c>
-      <c r="C6" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A6,'Casos de teste'!$K$2:$K$66,"Passou")</f>
+      <c r="A6" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$83,A6)</f>
+        <v>15</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A6,'Casos de teste'!$L$2:$L$83,"Passou")</f>
         <v>0</v>
       </c>
-      <c r="D6" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A6,'Casos de teste'!$K$2:$K$66,"Falhou")</f>
+      <c r="D6" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A6,'Casos de teste'!$L$2:$L$83,"Falhou")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A6,'Casos de teste'!$K$2:$K$66,"Bloqueado")</f>
+      <c r="E6" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A6,'Casos de teste'!$L$2:$L$83,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="F6" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A6,'Casos de teste'!$K$2:$K$66,"Não testado")</f>
-        <v>10</v>
-      </c>
-      <c r="G6" s="10" t="n">
+      <c r="F6" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A6,'Casos de teste'!$L$2:$L$83,"Não testado")</f>
+        <v>15</v>
+      </c>
+      <c r="G6" s="11" t="n">
         <f aca="false">IF(B6=0,0,(C6+D6)/B6)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="10" t="str">
+      <c r="H6" s="11" t="str">
         <f aca="false">IF(C6+D6=0,"-",C6/(C6+D6))</f>
         <v>-</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="B7" s="9" t="n">
-        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$66,A7)</f>
+      <c r="A7" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$83,A7)</f>
         <v>5</v>
       </c>
-      <c r="C7" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A7,'Casos de teste'!$K$2:$K$66,"Passou")</f>
+      <c r="C7" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A7,'Casos de teste'!$L$2:$L$83,"Passou")</f>
         <v>0</v>
       </c>
-      <c r="D7" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A7,'Casos de teste'!$K$2:$K$66,"Falhou")</f>
+      <c r="D7" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A7,'Casos de teste'!$L$2:$L$83,"Falhou")</f>
         <v>0</v>
       </c>
-      <c r="E7" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A7,'Casos de teste'!$K$2:$K$66,"Bloqueado")</f>
+      <c r="E7" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A7,'Casos de teste'!$L$2:$L$83,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="F7" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A7,'Casos de teste'!$K$2:$K$66,"Não testado")</f>
+      <c r="F7" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A7,'Casos de teste'!$L$2:$L$83,"Não testado")</f>
         <v>5</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="n">
         <f aca="false">IF(B7=0,0,(C7+D7)/B7)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="10" t="str">
+      <c r="H7" s="11" t="str">
         <f aca="false">IF(C7+D7=0,"-",C7/(C7+D7))</f>
         <v>-</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>302</v>
-      </c>
-      <c r="B8" s="9" t="n">
-        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$66,A8)</f>
+      <c r="A8" s="10" t="s">
+        <v>385</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$83,A8)</f>
         <v>6</v>
       </c>
-      <c r="C8" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A8,'Casos de teste'!$K$2:$K$66,"Passou")</f>
+      <c r="C8" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A8,'Casos de teste'!$L$2:$L$83,"Passou")</f>
         <v>0</v>
       </c>
-      <c r="D8" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A8,'Casos de teste'!$K$2:$K$66,"Falhou")</f>
+      <c r="D8" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A8,'Casos de teste'!$L$2:$L$83,"Falhou")</f>
         <v>0</v>
       </c>
-      <c r="E8" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A8,'Casos de teste'!$K$2:$K$66,"Bloqueado")</f>
+      <c r="E8" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A8,'Casos de teste'!$L$2:$L$83,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="F8" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A8,'Casos de teste'!$K$2:$K$66,"Não testado")</f>
+      <c r="F8" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A8,'Casos de teste'!$L$2:$L$83,"Não testado")</f>
         <v>6</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="11" t="n">
         <f aca="false">IF(B8=0,0,(C8+D8)/B8)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="10" t="str">
+      <c r="H8" s="11" t="str">
         <f aca="false">IF(C8+D8=0,"-",C8/(C8+D8))</f>
         <v>-</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>331</v>
-      </c>
-      <c r="B9" s="9" t="n">
-        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$66,A9)</f>
+      <c r="A9" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="B9" s="10" t="n">
+        <f aca="false">COUNTIF('Casos de teste'!$C$2:$C$83,A9)</f>
         <v>8</v>
       </c>
-      <c r="C9" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A9,'Casos de teste'!$K$2:$K$66,"Passou")</f>
+      <c r="C9" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A9,'Casos de teste'!$L$2:$L$83,"Passou")</f>
         <v>0</v>
       </c>
-      <c r="D9" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A9,'Casos de teste'!$K$2:$K$66,"Falhou")</f>
+      <c r="D9" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A9,'Casos de teste'!$L$2:$L$83,"Falhou")</f>
         <v>0</v>
       </c>
-      <c r="E9" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A9,'Casos de teste'!$K$2:$K$66,"Bloqueado")</f>
+      <c r="E9" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A9,'Casos de teste'!$L$2:$L$83,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="F9" s="9" t="n">
-        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$66,$A9,'Casos de teste'!$K$2:$K$66,"Não testado")</f>
+      <c r="F9" s="10" t="n">
+        <f aca="false">COUNTIFS('Casos de teste'!$C$2:$C$83,$A9,'Casos de teste'!$L$2:$L$83,"Não testado")</f>
         <v>8</v>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="11" t="n">
         <f aca="false">IF(B9=0,0,(C9+D9)/B9)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="10" t="str">
+      <c r="H9" s="11" t="str">
         <f aca="false">IF(C9+D9=0,"-",C9/(C9+D9))</f>
         <v>-</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>374</v>
-      </c>
-      <c r="B10" s="11" t="n">
+      <c r="A10" s="12" t="s">
+        <v>455</v>
+      </c>
+      <c r="B10" s="12" t="n">
         <f aca="false">SUM(B2:B9)</f>
-        <v>65</v>
-      </c>
-      <c r="C10" s="11" t="n">
+        <v>82</v>
+      </c>
+      <c r="C10" s="12" t="n">
         <f aca="false">SUM(C2:C9)</f>
         <v>1</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <f aca="false">SUM(D2:D9)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="12" t="n">
         <f aca="false">SUM(E2:E9)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <f aca="false">SUM(F2:F9)</f>
-        <v>64</v>
-      </c>
-      <c r="G10" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="G10" s="13" t="n">
         <f aca="false">IF(B10=0,0,(C10+D10)/B10)</f>
-        <v>0.0153846153846154</v>
-      </c>
-      <c r="H10" s="12" t="n">
+        <v>0.0121951219512195</v>
+      </c>
+      <c r="H10" s="13" t="n">
         <f aca="false">IF(C10+D10=0,"-",C10/(C10+D10))</f>
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>375</v>
+      <c r="A12" s="14" t="s">
+        <v>456</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>376</v>
-      </c>
-      <c r="B13" s="15" t="str">
-        <f aca="false" t="array" ref="B13:B13">IFERROR(_xlfn.TEXTJOIN(", ",TRUE(),IF('Casos de teste'!$K$2:$K$66="Falhou",'Casos de teste'!$A$2:$A$66,"")),"")</f>
+      <c r="A13" s="15" t="s">
+        <v>457</v>
+      </c>
+      <c r="B13" s="16" t="str">
+        <f aca="false" t="array" ref="B13:B13">IFERROR(_xlfn.TEXTJOIN(", ",TRUE(),IF('Casos de teste'!$L$2:$L$83="Falhou",'Casos de teste'!$A$2:$A$83,"")),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>